<commit_message>
demoted dev test to draft
</commit_message>
<xml_diff>
--- a/docs/Website-Events.xlsx
+++ b/docs/Website-Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39638bab59bf7aaa/Projects/shpe-uwm/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_2B20284E939059CB5C7D0A5E0D70175D97735ACC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EFAD8B5-48FF-40DB-B942-0269C83578D3}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_2B20284E939059CB5C7D0A5E0D70175D97735ACC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AFA37AB-FE38-4828-A43F-1ED972644C6B}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15634" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -456,7 +456,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EventsTable" displayName="EventsTable" ref="A7:H28" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EventsTable" displayName="EventsTable" ref="A7:H52" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Status"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Event ID"/>

</xml_diff>